<commit_message>
Update portfolio infographics and documents
</commit_message>
<xml_diff>
--- a/public/e5-tableau-synthese-2026.xlsx
+++ b/public/e5-tableau-synthese-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vspir\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programming\!portfolio\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13EA2B01-8D2A-40C2-8922-D34322D0AFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76AE2D2-A307-414E-8C6B-E78EA4409FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -140,9 +140,6 @@
     <t>du 04/11/2024 au 04/11/2024</t>
   </si>
   <si>
-    <t>du 01/11/2024 au 6/11/2024</t>
-  </si>
-  <si>
     <t>du 15/12/2024 au 06/01/2025</t>
   </si>
   <si>
@@ -152,9 +149,6 @@
     <t>du 24/2/202 au 31/07/2026</t>
   </si>
   <si>
-    <t>du 08/10/2024 au 8/10/2024</t>
-  </si>
-  <si>
     <t>du 14/11/2024 au 6/07/2025</t>
   </si>
   <si>
@@ -167,9 +161,6 @@
     <t>du 02/12/2025 au 31/07/2026</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio : https://www.spirine.fyi/</t>
-  </si>
-  <si>
     <t>Réponses aux tickets des clients</t>
   </si>
   <si>
@@ -189,6 +180,15 @@
   </si>
   <si>
     <t>Création d'un site de recherche de coéquipiers pour des jeux avec mes camarades</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://www.spirine.fyi</t>
+  </si>
+  <si>
+    <t>du 08/10/2024 au 25/10/2025</t>
+  </si>
+  <si>
+    <t>du 01/11/2024 au 06/11/2024</t>
   </si>
 </sst>
 </file>
@@ -732,15 +732,45 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -773,36 +803,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1149,30 +1149,30 @@
       <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="44" t="s">
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="39"/>
-      <c r="H3" s="45"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="34"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
       <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
@@ -1184,22 +1184,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
+      <c r="A5" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="43" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1222,8 +1222,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25"/>
-      <c r="B7" s="34"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="15" t="s">
         <v>9</v>
       </c>
@@ -1279,16 +1279,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="39"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1329,7 +1329,7 @@
       <c r="A9" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="24" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="17"/>
@@ -1378,10 +1378,10 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="47" t="s">
-        <v>32</v>
+        <v>43</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>48</v>
       </c>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
@@ -1429,10 +1429,10 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B11" s="47" t="s">
-        <v>33</v>
+        <v>44</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>32</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
@@ -1482,8 +1482,8 @@
       <c r="A12" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="47" t="s">
-        <v>34</v>
+      <c r="B12" s="25" t="s">
+        <v>33</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
@@ -1533,8 +1533,8 @@
       <c r="A13" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="47" t="s">
-        <v>36</v>
+      <c r="B13" s="25" t="s">
+        <v>47</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>29</v>
@@ -1586,8 +1586,8 @@
       <c r="A14" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="47" t="s">
-        <v>35</v>
+      <c r="B14" s="25" t="s">
+        <v>34</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
@@ -1635,10 +1635,10 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="47" t="s">
-        <v>37</v>
+        <v>45</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>35</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
@@ -1822,16 +1822,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="32"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="42"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1870,10 +1870,10 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="46" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>36</v>
       </c>
       <c r="C20" s="16"/>
       <c r="D20" s="16" t="s">
@@ -1923,10 +1923,10 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="46" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>36</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>29</v>
@@ -1976,10 +1976,10 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="46" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="B22" s="24" t="s">
+        <v>37</v>
       </c>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
@@ -2206,16 +2206,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="32"/>
+      <c r="B27" s="41"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="41"/>
+      <c r="H27" s="42"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2254,10 +2254,10 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>38</v>
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
@@ -2305,10 +2305,10 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B29" s="46" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>36</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>29</v>
@@ -2358,10 +2358,10 @@
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B30" s="46" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>37</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
@@ -2680,11 +2680,6 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2692,6 +2687,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>